<commit_message>
Updated notebooks and figures for the paper
</commit_message>
<xml_diff>
--- a/results/skill/2021_2022/compare_results_2021_2022.xlsx
+++ b/results/skill/2021_2022/compare_results_2021_2022.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\casadje\GitHub\EFAS_skill\results\skill\2021_2022\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD26A396-796D-45C6-8DE3-9F4B18C19256}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB89BDCC-9CB3-4F8A-8374-9C259148977D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12810" tabRatio="795" activeTab="1" xr2:uid="{4001A787-8C98-4466-95B5-A97BAB92B13F}"/>
   </bookViews>
@@ -1981,16 +1981,6 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EDF4A9CD-DC66-4780-9A13-6AACFBE5CE57}" name="skill_by_criteria__243" displayName="skill_by_criteria__243" ref="A1:Q117" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:Q117" xr:uid="{195E5C6F-BE29-47EF-8AE5-2414E38EAF89}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="EUE"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="3">
-      <filters>
-        <filter val="f0.8"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="4">
       <filters>
         <filter val="60"/>
@@ -2002,6 +1992,9 @@
       </filters>
     </filterColumn>
   </autoFilter>
+  <sortState ref="A27:Q59">
+    <sortCondition ref="A1:A117"/>
+  </sortState>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{69C7BAED-ECE0-461B-BC7A-751D89958422}" uniqueName="1" name="approach/model" queryTableFieldId="1" dataDxfId="12"/>
     <tableColumn id="2" xr3:uid="{D1B0C460-FC1C-479D-920B-C8214A32D3AB}" uniqueName="2" name="window" queryTableFieldId="2"/>
@@ -2324,13 +2317,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24CE5352-E4DB-4452-A238-93008838F217}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:O97"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.1796875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>29</v>
       </c>
@@ -2377,7 +2370,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
         <v>3</v>
       </c>
@@ -2424,7 +2417,7 @@
         <v>0.44700000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
         <v>3</v>
       </c>
@@ -2469,7 +2462,7 @@
         <v>0.436</v>
       </c>
     </row>
-    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
         <v>3</v>
       </c>
@@ -2516,7 +2509,7 @@
         <v>0.45200000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="11" t="s">
         <v>3</v>
       </c>
@@ -2561,7 +2554,7 @@
         <v>0.441</v>
       </c>
     </row>
-    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
         <v>3</v>
       </c>
@@ -2608,7 +2601,7 @@
         <v>0.45200000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>3</v>
       </c>
@@ -2653,7 +2646,7 @@
         <v>0.44400000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="16" t="s">
         <v>3</v>
       </c>
@@ -2698,7 +2691,7 @@
         <v>0.47299999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="16" t="s">
         <v>3</v>
       </c>
@@ -2741,7 +2734,7 @@
         <v>0.45700000000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="16" t="s">
         <v>3</v>
       </c>
@@ -2786,7 +2779,7 @@
         <v>0.48499999999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="16" t="s">
         <v>3</v>
       </c>
@@ -2829,7 +2822,7 @@
         <v>0.47099999999999997</v>
       </c>
     </row>
-    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="16" t="s">
         <v>3</v>
       </c>
@@ -2874,7 +2867,7 @@
         <v>0.52200000000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="16" t="s">
         <v>3</v>
       </c>
@@ -2917,7 +2910,7 @@
         <v>0.48199999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="16" t="s">
         <v>3</v>
       </c>
@@ -2962,7 +2955,7 @@
         <v>0.505</v>
       </c>
     </row>
-    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="16" t="s">
         <v>3</v>
       </c>
@@ -3005,7 +2998,7 @@
         <v>0.48799999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="16" t="s">
         <v>3</v>
       </c>
@@ -3050,7 +3043,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="17" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="16" t="s">
         <v>3</v>
       </c>
@@ -3093,7 +3086,7 @@
         <v>0.503</v>
       </c>
     </row>
-    <row r="18" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="16" t="s">
         <v>3</v>
       </c>
@@ -3138,7 +3131,7 @@
         <v>0.52200000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="16" t="s">
         <v>3</v>
       </c>
@@ -3181,7 +3174,7 @@
         <v>0.505</v>
       </c>
     </row>
-    <row r="20" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="16" t="s">
         <v>3</v>
       </c>
@@ -3226,7 +3219,7 @@
         <v>0.50900000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="16" t="s">
         <v>3</v>
       </c>
@@ -3269,7 +3262,7 @@
         <v>0.48799999999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="16" t="s">
         <v>3</v>
       </c>
@@ -3314,7 +3307,7 @@
         <v>0.52400000000000002</v>
       </c>
     </row>
-    <row r="23" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="16" t="s">
         <v>3</v>
       </c>
@@ -3357,7 +3350,7 @@
         <v>0.503</v>
       </c>
     </row>
-    <row r="24" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="16" t="s">
         <v>3</v>
       </c>
@@ -3402,7 +3395,7 @@
         <v>0.52400000000000002</v>
       </c>
     </row>
-    <row r="25" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="16" t="s">
         <v>3</v>
       </c>
@@ -3445,7 +3438,7 @@
         <v>0.505</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A26" s="16" t="s">
         <v>16</v>
       </c>
@@ -3490,7 +3483,7 @@
         <v>0.45200000000000001</v>
       </c>
     </row>
-    <row r="27" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="16" t="s">
         <v>16</v>
       </c>
@@ -3533,7 +3526,7 @@
         <v>0.443</v>
       </c>
     </row>
-    <row r="28" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="16" t="s">
         <v>16</v>
       </c>
@@ -3578,7 +3571,7 @@
         <v>0.46600000000000003</v>
       </c>
     </row>
-    <row r="29" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="16" t="s">
         <v>16</v>
       </c>
@@ -3621,7 +3614,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="30" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="16" t="s">
         <v>16</v>
       </c>
@@ -3666,7 +3659,7 @@
         <v>0.46200000000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="16" t="s">
         <v>16</v>
       </c>
@@ -3709,7 +3702,7 @@
         <v>0.45200000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="16" t="s">
         <v>16</v>
       </c>
@@ -3756,7 +3749,7 @@
         <v>0.47399999999999998</v>
       </c>
     </row>
-    <row r="33" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="16" t="s">
         <v>16</v>
       </c>
@@ -3799,7 +3792,7 @@
         <v>0.443</v>
       </c>
     </row>
-    <row r="34" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="16" t="s">
         <v>16</v>
       </c>
@@ -3844,7 +3837,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="35" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="16" t="s">
         <v>16</v>
       </c>
@@ -3887,7 +3880,7 @@
         <v>0.47899999999999998</v>
       </c>
     </row>
-    <row r="36" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="16" t="s">
         <v>16</v>
       </c>
@@ -3932,7 +3925,7 @@
         <v>0.495</v>
       </c>
     </row>
-    <row r="37" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="16" t="s">
         <v>16</v>
       </c>
@@ -3975,7 +3968,7 @@
         <v>0.48699999999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="16" t="s">
         <v>16</v>
       </c>
@@ -4022,7 +4015,7 @@
         <v>0.47399999999999998</v>
       </c>
     </row>
-    <row r="39" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="16" t="s">
         <v>16</v>
       </c>
@@ -4065,7 +4058,7 @@
         <v>0.45900000000000002</v>
       </c>
     </row>
-    <row r="40" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="16" t="s">
         <v>16</v>
       </c>
@@ -4110,7 +4103,7 @@
         <v>0.49299999999999999</v>
       </c>
     </row>
-    <row r="41" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="16" t="s">
         <v>16</v>
       </c>
@@ -4153,7 +4146,7 @@
         <v>0.47799999999999998</v>
       </c>
     </row>
-    <row r="42" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="16" t="s">
         <v>16</v>
       </c>
@@ -4198,7 +4191,7 @@
         <v>0.504</v>
       </c>
     </row>
-    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="16" t="s">
         <v>16</v>
       </c>
@@ -4241,7 +4234,7 @@
         <v>0.48699999999999999</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A44" s="16" t="s">
         <v>17</v>
       </c>
@@ -4288,7 +4281,7 @@
         <v>0.434</v>
       </c>
     </row>
-    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="16" t="s">
         <v>17</v>
       </c>
@@ -4333,7 +4326,7 @@
         <v>0.41499999999999998</v>
       </c>
     </row>
-    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="16" t="s">
         <v>17</v>
       </c>
@@ -4380,7 +4373,7 @@
         <v>0.443</v>
       </c>
     </row>
-    <row r="47" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="16" t="s">
         <v>17</v>
       </c>
@@ -4423,7 +4416,7 @@
         <v>0.41099999999999998</v>
       </c>
     </row>
-    <row r="48" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="16" t="s">
         <v>17</v>
       </c>
@@ -4470,7 +4463,7 @@
         <v>0.45100000000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="16" t="s">
         <v>17</v>
       </c>
@@ -4515,7 +4508,7 @@
         <v>0.436</v>
       </c>
     </row>
-    <row r="50" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="16" t="s">
         <v>17</v>
       </c>
@@ -4562,7 +4555,7 @@
         <v>0.46800000000000003</v>
       </c>
     </row>
-    <row r="51" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="16" t="s">
         <v>17</v>
       </c>
@@ -4607,7 +4600,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="52" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="16" t="s">
         <v>17</v>
       </c>
@@ -4654,7 +4647,7 @@
         <v>0.48699999999999999</v>
       </c>
     </row>
-    <row r="53" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="16" t="s">
         <v>17</v>
       </c>
@@ -4699,7 +4692,7 @@
         <v>0.47499999999999998</v>
       </c>
     </row>
-    <row r="54" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="16" t="s">
         <v>17</v>
       </c>
@@ -4746,7 +4739,7 @@
         <v>0.49299999999999999</v>
       </c>
     </row>
-    <row r="55" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="16" t="s">
         <v>17</v>
       </c>
@@ -4791,7 +4784,7 @@
         <v>0.48499999999999999</v>
       </c>
     </row>
-    <row r="56" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="16" t="s">
         <v>17</v>
       </c>
@@ -4838,7 +4831,7 @@
         <v>0.46899999999999997</v>
       </c>
     </row>
-    <row r="57" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="16" t="s">
         <v>17</v>
       </c>
@@ -4883,7 +4876,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="58" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="16" t="s">
         <v>17</v>
       </c>
@@ -4930,7 +4923,7 @@
         <v>0.48699999999999999</v>
       </c>
     </row>
-    <row r="59" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="16" t="s">
         <v>17</v>
       </c>
@@ -4975,7 +4968,7 @@
         <v>0.47499999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="16" t="s">
         <v>17</v>
       </c>
@@ -5022,7 +5015,7 @@
         <v>0.49299999999999999</v>
       </c>
     </row>
-    <row r="61" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="16" t="s">
         <v>17</v>
       </c>
@@ -5067,7 +5060,7 @@
         <v>0.48499999999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A62" s="16" t="s">
         <v>2</v>
       </c>
@@ -5112,7 +5105,7 @@
         <v>0.48899999999999999</v>
       </c>
     </row>
-    <row r="63" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="16" t="s">
         <v>2</v>
       </c>
@@ -5155,7 +5148,7 @@
         <v>0.45800000000000002</v>
       </c>
     </row>
-    <row r="64" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="16" t="s">
         <v>2</v>
       </c>
@@ -5200,7 +5193,7 @@
         <v>0.46600000000000003</v>
       </c>
     </row>
-    <row r="65" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="16" t="s">
         <v>2</v>
       </c>
@@ -5243,7 +5236,7 @@
         <v>0.46700000000000003</v>
       </c>
     </row>
-    <row r="66" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="16" t="s">
         <v>2</v>
       </c>
@@ -5288,7 +5281,7 @@
         <v>0.498</v>
       </c>
     </row>
-    <row r="67" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="16" t="s">
         <v>2</v>
       </c>
@@ -5331,7 +5324,7 @@
         <v>0.47099999999999997</v>
       </c>
     </row>
-    <row r="68" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="16" t="s">
         <v>2</v>
       </c>
@@ -5376,7 +5369,7 @@
         <v>0.48899999999999999</v>
       </c>
     </row>
-    <row r="69" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="16" t="s">
         <v>2</v>
       </c>
@@ -5419,7 +5412,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="70" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="16" t="s">
         <v>2</v>
       </c>
@@ -5464,7 +5457,7 @@
         <v>0.49299999999999999</v>
       </c>
     </row>
-    <row r="71" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="16" t="s">
         <v>2</v>
       </c>
@@ -5507,7 +5500,7 @@
         <v>0.47899999999999998</v>
       </c>
     </row>
-    <row r="72" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="16" t="s">
         <v>2</v>
       </c>
@@ -5552,7 +5545,7 @@
         <v>0.498</v>
       </c>
     </row>
-    <row r="73" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="16" t="s">
         <v>2</v>
       </c>
@@ -5595,7 +5588,7 @@
         <v>0.48199999999999998</v>
       </c>
     </row>
-    <row r="74" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="16" t="s">
         <v>2</v>
       </c>
@@ -5640,7 +5633,7 @@
         <v>0.48599999999999999</v>
       </c>
     </row>
-    <row r="75" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="16" t="s">
         <v>2</v>
       </c>
@@ -5683,7 +5676,7 @@
         <v>0.46899999999999997</v>
       </c>
     </row>
-    <row r="76" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="16" t="s">
         <v>2</v>
       </c>
@@ -5728,7 +5721,7 @@
         <v>0.49399999999999999</v>
       </c>
     </row>
-    <row r="77" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="16" t="s">
         <v>2</v>
       </c>
@@ -5772,7 +5765,7 @@
         <v>0.47893944395074262</v>
       </c>
     </row>
-    <row r="78" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="16" t="s">
         <v>2</v>
       </c>
@@ -5820,7 +5813,7 @@
         <v>0.5101637548119633</v>
       </c>
     </row>
-    <row r="79" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="16" t="s">
         <v>2</v>
       </c>
@@ -5866,7 +5859,7 @@
         <v>0.48884755738669805</v>
       </c>
     </row>
-    <row r="80" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>23</v>
       </c>
@@ -5910,7 +5903,7 @@
         <v>0.45700000000000002</v>
       </c>
     </row>
-    <row r="81" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>23</v>
       </c>
@@ -5954,7 +5947,7 @@
         <v>0.45700000000000002</v>
       </c>
     </row>
-    <row r="82" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>23</v>
       </c>
@@ -5998,7 +5991,7 @@
         <v>0.45800000000000002</v>
       </c>
     </row>
-    <row r="83" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>24</v>
       </c>
@@ -6042,7 +6035,7 @@
         <v>0.42899999999999999</v>
       </c>
     </row>
-    <row r="84" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>24</v>
       </c>
@@ -6086,7 +6079,7 @@
         <v>0.437</v>
       </c>
     </row>
-    <row r="85" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>24</v>
       </c>
@@ -6130,7 +6123,7 @@
         <v>0.44600000000000001</v>
       </c>
     </row>
-    <row r="86" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>21</v>
       </c>
@@ -6174,7 +6167,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="87" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>21</v>
       </c>
@@ -6218,7 +6211,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="88" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>21</v>
       </c>
@@ -6262,7 +6255,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="89" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>22</v>
       </c>
@@ -6306,7 +6299,7 @@
         <v>0.44700000000000001</v>
       </c>
     </row>
-    <row r="90" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>22</v>
       </c>
@@ -6350,7 +6343,7 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="91" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:15" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>22</v>
       </c>
@@ -6394,17 +6387,17 @@
         <v>0.48199999999999998</v>
       </c>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A95" s="26" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A96" s="25" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A97" s="33" t="s">
         <v>30</v>
       </c>
@@ -6630,15 +6623,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{981285E5-5B1F-4ECD-8D9D-A8A24790817E}">
   <dimension ref="A1:S149"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="9.140625" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="9.140625" customWidth="1"/>
-    <col min="16" max="17" width="0" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="9.1796875" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="9.1796875" customWidth="1"/>
+    <col min="16" max="17" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -6691,7 +6684,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="34" t="s">
         <v>3</v>
       </c>
@@ -6744,7 +6737,7 @@
         <v>0.56299999999999994</v>
       </c>
     </row>
-    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="21" t="s">
         <v>3</v>
       </c>
@@ -6795,7 +6788,7 @@
         <v>0.66800000000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="21" t="s">
         <v>16</v>
       </c>
@@ -6846,7 +6839,7 @@
         <v>0.67400000000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="21" t="s">
         <v>23</v>
       </c>
@@ -6897,7 +6890,7 @@
         <v>0.66600000000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="21" t="s">
         <v>24</v>
       </c>
@@ -6948,7 +6941,7 @@
         <v>0.55400000000000005</v>
       </c>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="21" t="s">
         <v>21</v>
       </c>
@@ -6999,7 +6992,7 @@
         <v>0.58799999999999997</v>
       </c>
     </row>
-    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="21" t="s">
         <v>22</v>
       </c>
@@ -7050,7 +7043,7 @@
         <v>0.68100000000000005</v>
       </c>
     </row>
-    <row r="9" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="21" t="s">
         <v>17</v>
       </c>
@@ -7101,7 +7094,7 @@
         <v>0.67500000000000004</v>
       </c>
     </row>
-    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="21" t="s">
         <v>2</v>
       </c>
@@ -7152,7 +7145,7 @@
         <v>0.67600000000000005</v>
       </c>
     </row>
-    <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="21" t="s">
         <v>3</v>
       </c>
@@ -7203,7 +7196,7 @@
         <v>0.66800000000000004</v>
       </c>
     </row>
-    <row r="12" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="21" t="s">
         <v>16</v>
       </c>
@@ -7254,7 +7247,7 @@
         <v>0.67400000000000004</v>
       </c>
     </row>
-    <row r="13" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="21" t="s">
         <v>23</v>
       </c>
@@ -7305,7 +7298,7 @@
         <v>0.66600000000000004</v>
       </c>
     </row>
-    <row r="14" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="21" t="s">
         <v>24</v>
       </c>
@@ -7354,7 +7347,7 @@
         <v>0.59799999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="21" t="s">
         <v>21</v>
       </c>
@@ -7403,7 +7396,7 @@
         <v>0.63100000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="21" t="s">
         <v>22</v>
       </c>
@@ -7454,7 +7447,7 @@
         <v>0.68100000000000005</v>
       </c>
     </row>
-    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="21" t="s">
         <v>17</v>
       </c>
@@ -7505,7 +7498,7 @@
         <v>0.67500000000000004</v>
       </c>
     </row>
-    <row r="18" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="21" t="s">
         <v>2</v>
       </c>
@@ -7556,7 +7549,7 @@
         <v>0.67600000000000005</v>
       </c>
     </row>
-    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="21" t="s">
         <v>3</v>
       </c>
@@ -7607,7 +7600,7 @@
         <v>0.66800000000000004</v>
       </c>
     </row>
-    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="21" t="s">
         <v>16</v>
       </c>
@@ -7658,7 +7651,7 @@
         <v>0.67400000000000004</v>
       </c>
     </row>
-    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="21" t="s">
         <v>17</v>
       </c>
@@ -7709,7 +7702,7 @@
         <v>0.67500000000000004</v>
       </c>
     </row>
-    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="21" t="s">
         <v>2</v>
       </c>
@@ -7760,7 +7753,7 @@
         <v>0.67800000000000005</v>
       </c>
     </row>
-    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="21" t="s">
         <v>23</v>
       </c>
@@ -7811,7 +7804,7 @@
         <v>0.66800000000000004</v>
       </c>
     </row>
-    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="21" t="s">
         <v>24</v>
       </c>
@@ -7860,7 +7853,7 @@
         <v>0.59799999999999998</v>
       </c>
     </row>
-    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="21" t="s">
         <v>21</v>
       </c>
@@ -7909,7 +7902,7 @@
         <v>0.63100000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="21" t="s">
         <v>22</v>
       </c>
@@ -7960,7 +7953,7 @@
         <v>0.68100000000000005</v>
       </c>
     </row>
-    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A27" s="34" t="s">
         <v>3</v>
       </c>
@@ -8013,7 +8006,7 @@
         <v>0.441</v>
       </c>
     </row>
-    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="34" t="s">
         <v>3</v>
       </c>
@@ -8066,7 +8059,7 @@
         <v>0.439</v>
       </c>
     </row>
-    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A29" s="21" t="s">
         <v>3</v>
       </c>
@@ -8117,7 +8110,7 @@
         <v>0.48899999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="21" t="s">
         <v>3</v>
       </c>
@@ -8168,9 +8161,9 @@
         <v>0.48699999999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A31" s="21" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="B31">
         <v>1</v>
@@ -8179,7 +8172,7 @@
         <v>0.5</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E31">
         <v>60</v>
@@ -8188,38 +8181,38 @@
         <v>132</v>
       </c>
       <c r="G31" s="1">
-        <v>0.57499999999999996</v>
+        <v>0.4</v>
       </c>
       <c r="H31" s="21"/>
       <c r="I31" s="7">
-        <v>279</v>
+        <v>339</v>
       </c>
       <c r="J31" s="7">
-        <v>399</v>
+        <v>339</v>
       </c>
       <c r="K31" s="7">
-        <v>172</v>
+        <v>318</v>
       </c>
       <c r="L31" s="8">
         <v>678</v>
       </c>
-      <c r="M31" s="36">
-        <v>0.41199999999999998</v>
+      <c r="M31" s="9">
+        <v>0.5</v>
       </c>
       <c r="N31" s="9">
-        <v>0.61899999999999999</v>
+        <v>0.51600000000000001</v>
       </c>
       <c r="O31" s="9">
-        <v>0.51700000000000002</v>
-      </c>
-      <c r="P31" s="36">
-        <v>0.49399999999999999</v>
-      </c>
-      <c r="Q31" s="36">
-        <v>0.47299999999999998</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.51</v>
+      </c>
+      <c r="P31" s="9">
+        <v>0.50800000000000001</v>
+      </c>
+      <c r="Q31" s="9">
+        <v>0.50600000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="21" t="s">
         <v>16</v>
       </c>
@@ -8270,9 +8263,9 @@
         <v>0.443</v>
       </c>
     </row>
-    <row r="33" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A33" s="21" t="s">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="B33">
         <v>1</v>
@@ -8281,7 +8274,7 @@
         <v>0.5</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="E33">
         <v>60</v>
@@ -8290,38 +8283,38 @@
         <v>132</v>
       </c>
       <c r="G33" s="1">
-        <v>0.52500000000000002</v>
+        <v>0.35</v>
       </c>
       <c r="H33" s="21"/>
       <c r="I33" s="7">
-        <v>273</v>
+        <v>355</v>
       </c>
       <c r="J33" s="7">
-        <v>405</v>
+        <v>323</v>
       </c>
       <c r="K33" s="7">
-        <v>200</v>
+        <v>370</v>
       </c>
       <c r="L33" s="8">
         <v>678</v>
       </c>
       <c r="M33" s="9">
-        <v>0.40300000000000002</v>
+        <v>0.52400000000000002</v>
       </c>
       <c r="N33" s="9">
-        <v>0.57699999999999996</v>
+        <v>0.49</v>
       </c>
       <c r="O33" s="9">
-        <v>0.49399999999999999</v>
+        <v>0.502</v>
       </c>
       <c r="P33" s="9">
-        <v>0.47399999999999998</v>
+        <v>0.50600000000000001</v>
       </c>
       <c r="Q33" s="9">
-        <v>0.45700000000000002</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="21" t="s">
         <v>23</v>
       </c>
@@ -8372,9 +8365,9 @@
         <v>0.45700000000000002</v>
       </c>
     </row>
-    <row r="35" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A35" s="21" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B35">
         <v>1</v>
@@ -8391,41 +8384,41 @@
       <c r="F35">
         <v>132</v>
       </c>
-      <c r="G35" s="1"/>
-      <c r="H35" s="21" t="s">
-        <v>10</v>
-      </c>
+      <c r="G35" s="1">
+        <v>0.57499999999999996</v>
+      </c>
+      <c r="H35" s="21"/>
       <c r="I35" s="7">
-        <v>263</v>
+        <v>279</v>
       </c>
       <c r="J35" s="7">
-        <v>415</v>
+        <v>399</v>
       </c>
       <c r="K35" s="7">
-        <v>245</v>
+        <v>172</v>
       </c>
       <c r="L35" s="8">
         <v>678</v>
       </c>
-      <c r="M35" s="9">
-        <v>0.38800000000000001</v>
+      <c r="M35" s="36">
+        <v>0.41199999999999998</v>
       </c>
       <c r="N35" s="9">
-        <v>0.51800000000000002</v>
+        <v>0.61899999999999999</v>
       </c>
       <c r="O35" s="9">
-        <v>0.45800000000000002</v>
-      </c>
-      <c r="P35" s="9">
-        <v>0.44400000000000001</v>
-      </c>
-      <c r="Q35" s="9">
-        <v>0.43</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.51700000000000002</v>
+      </c>
+      <c r="P35" s="36">
+        <v>0.49399999999999999</v>
+      </c>
+      <c r="Q35" s="36">
+        <v>0.47299999999999998</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A36" s="21" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="B36">
         <v>1</v>
@@ -8443,38 +8436,38 @@
         <v>132</v>
       </c>
       <c r="G36" s="1">
-        <v>0.4</v>
+        <v>0.57499999999999996</v>
       </c>
       <c r="H36" s="21"/>
       <c r="I36" s="7">
-        <v>339</v>
+        <v>279</v>
       </c>
       <c r="J36" s="7">
-        <v>339</v>
+        <v>399</v>
       </c>
       <c r="K36" s="7">
-        <v>318</v>
+        <v>172</v>
       </c>
       <c r="L36" s="8">
         <v>678</v>
       </c>
       <c r="M36" s="9">
-        <v>0.5</v>
+        <v>0.41199999999999998</v>
       </c>
       <c r="N36" s="9">
-        <v>0.51600000000000001</v>
+        <v>0.61899999999999999</v>
       </c>
       <c r="O36" s="9">
-        <v>0.51</v>
+        <v>0.51700000000000002</v>
       </c>
       <c r="P36" s="9">
-        <v>0.50800000000000001</v>
+        <v>0.49399999999999999</v>
       </c>
       <c r="Q36" s="9">
-        <v>0.50600000000000001</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.47299999999999998</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A37" s="21" t="s">
         <v>16</v>
       </c>
@@ -8485,7 +8478,7 @@
         <v>0.5</v>
       </c>
       <c r="D37" s="21" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="E37">
         <v>60</v>
@@ -8494,38 +8487,38 @@
         <v>132</v>
       </c>
       <c r="G37" s="1">
-        <v>0.57499999999999996</v>
+        <v>0.35</v>
       </c>
       <c r="H37" s="21"/>
       <c r="I37" s="7">
-        <v>279</v>
+        <v>360</v>
       </c>
       <c r="J37" s="7">
-        <v>399</v>
+        <v>318</v>
       </c>
       <c r="K37" s="7">
-        <v>172</v>
+        <v>440</v>
       </c>
       <c r="L37" s="8">
         <v>678</v>
       </c>
       <c r="M37" s="9">
-        <v>0.41199999999999998</v>
+        <v>0.53100000000000003</v>
       </c>
       <c r="N37" s="9">
-        <v>0.61899999999999999</v>
+        <v>0.45</v>
       </c>
       <c r="O37" s="9">
-        <v>0.51700000000000002</v>
+        <v>0.47799999999999998</v>
       </c>
       <c r="P37" s="9">
-        <v>0.49399999999999999</v>
+        <v>0.48699999999999999</v>
       </c>
       <c r="Q37" s="9">
-        <v>0.47299999999999998</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.496</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A38" s="21" t="s">
         <v>23</v>
       </c>
@@ -8536,7 +8529,7 @@
         <v>0.5</v>
       </c>
       <c r="D38" s="21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E38">
         <v>60</v>
@@ -8576,9 +8569,9 @@
         <v>0.45700000000000002</v>
       </c>
     </row>
-    <row r="39" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A39" s="21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B39">
         <v>1</v>
@@ -8595,41 +8588,41 @@
       <c r="F39">
         <v>132</v>
       </c>
-      <c r="G39" s="1"/>
-      <c r="H39" s="21" t="s">
-        <v>26</v>
-      </c>
+      <c r="G39" s="1">
+        <v>0.52500000000000002</v>
+      </c>
+      <c r="H39" s="21"/>
       <c r="I39" s="7">
-        <v>331</v>
+        <v>273</v>
       </c>
       <c r="J39" s="7">
-        <v>347</v>
+        <v>405</v>
       </c>
       <c r="K39" s="7">
-        <v>471</v>
+        <v>200</v>
       </c>
       <c r="L39" s="8">
         <v>678</v>
       </c>
       <c r="M39" s="9">
-        <v>0.48799999999999999</v>
+        <v>0.40300000000000002</v>
       </c>
       <c r="N39" s="9">
-        <v>0.41299999999999998</v>
+        <v>0.57699999999999996</v>
       </c>
       <c r="O39" s="9">
-        <v>0.439</v>
+        <v>0.49399999999999999</v>
       </c>
       <c r="P39" s="9">
-        <v>0.44700000000000001</v>
+        <v>0.47399999999999998</v>
       </c>
       <c r="Q39" s="9">
-        <v>0.45600000000000002</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.45700000000000002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A40" s="21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B40">
         <v>1</v>
@@ -8638,7 +8631,7 @@
         <v>0.5</v>
       </c>
       <c r="D40" s="21" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="E40">
         <v>60</v>
@@ -8646,41 +8639,41 @@
       <c r="F40">
         <v>132</v>
       </c>
-      <c r="G40" s="1"/>
-      <c r="H40" s="21" t="s">
-        <v>10</v>
-      </c>
+      <c r="G40" s="1">
+        <v>0.375</v>
+      </c>
+      <c r="H40" s="21"/>
       <c r="I40" s="7">
-        <v>248</v>
+        <v>324</v>
       </c>
       <c r="J40" s="7">
-        <v>430</v>
+        <v>354</v>
       </c>
       <c r="K40" s="7">
-        <v>187</v>
+        <v>428</v>
       </c>
       <c r="L40" s="8">
         <v>678</v>
       </c>
       <c r="M40" s="9">
-        <v>0.36599999999999999</v>
+        <v>0.47799999999999998</v>
       </c>
       <c r="N40" s="9">
-        <v>0.56999999999999995</v>
+        <v>0.43099999999999999</v>
       </c>
       <c r="O40" s="9">
-        <v>0.46800000000000003</v>
+        <v>0.44800000000000001</v>
       </c>
       <c r="P40" s="9">
-        <v>0.44600000000000001</v>
+        <v>0.45300000000000001</v>
       </c>
       <c r="Q40" s="9">
-        <v>0.42499999999999999</v>
-      </c>
-    </row>
-    <row r="41" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.45800000000000002</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A41" s="21" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B41">
         <v>1</v>
@@ -8689,7 +8682,7 @@
         <v>0.5</v>
       </c>
       <c r="D41" s="21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E41">
         <v>60</v>
@@ -8697,41 +8690,41 @@
       <c r="F41">
         <v>132</v>
       </c>
-      <c r="G41" s="1">
-        <v>0.4</v>
-      </c>
-      <c r="H41" s="21"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="21" t="s">
+        <v>10</v>
+      </c>
       <c r="I41" s="7">
-        <v>305</v>
+        <v>263</v>
       </c>
       <c r="J41" s="7">
-        <v>373</v>
+        <v>415</v>
       </c>
       <c r="K41" s="7">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="L41" s="8">
         <v>678</v>
       </c>
       <c r="M41" s="9">
-        <v>0.45</v>
+        <v>0.38800000000000001</v>
       </c>
       <c r="N41" s="9">
-        <v>0.56699999999999995</v>
+        <v>0.51800000000000002</v>
       </c>
       <c r="O41" s="9">
-        <v>0.51500000000000001</v>
+        <v>0.45800000000000002</v>
       </c>
       <c r="P41" s="9">
-        <v>0.502</v>
+        <v>0.44400000000000001</v>
       </c>
       <c r="Q41" s="9">
-        <v>0.48899999999999999</v>
-      </c>
-    </row>
-    <row r="42" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A42" s="21" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B42">
         <v>1</v>
@@ -8748,41 +8741,41 @@
       <c r="F42">
         <v>132</v>
       </c>
-      <c r="G42" s="1">
-        <v>0.4</v>
-      </c>
-      <c r="H42" s="21"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="21" t="s">
+        <v>26</v>
+      </c>
       <c r="I42" s="7">
-        <v>345</v>
+        <v>331</v>
       </c>
       <c r="J42" s="7">
-        <v>333</v>
+        <v>347</v>
       </c>
       <c r="K42" s="7">
-        <v>386</v>
+        <v>471</v>
       </c>
       <c r="L42" s="8">
         <v>678</v>
       </c>
       <c r="M42" s="9">
-        <v>0.50900000000000001</v>
+        <v>0.48799999999999999</v>
       </c>
       <c r="N42" s="9">
-        <v>0.47199999999999998</v>
+        <v>0.41299999999999998</v>
       </c>
       <c r="O42" s="9">
-        <v>0.48599999999999999</v>
+        <v>0.439</v>
       </c>
       <c r="P42" s="9">
-        <v>0.49</v>
+        <v>0.44700000000000001</v>
       </c>
       <c r="Q42" s="9">
-        <v>0.49399999999999999</v>
-      </c>
-    </row>
-    <row r="43" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.45600000000000002</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A43" s="21" t="s">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="B43">
         <v>1</v>
@@ -8791,7 +8784,7 @@
         <v>0.5</v>
       </c>
       <c r="D43" s="21" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="E43">
         <v>60</v>
@@ -8799,41 +8792,41 @@
       <c r="F43">
         <v>132</v>
       </c>
-      <c r="G43" s="1">
-        <v>0.25</v>
-      </c>
-      <c r="H43" s="21"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="21" t="s">
+        <v>26</v>
+      </c>
       <c r="I43" s="7">
-        <v>356</v>
+        <v>331</v>
       </c>
       <c r="J43" s="7">
-        <v>322</v>
+        <v>347</v>
       </c>
       <c r="K43" s="7">
-        <v>356</v>
+        <v>471</v>
       </c>
       <c r="L43" s="8">
         <v>678</v>
       </c>
       <c r="M43" s="9">
-        <v>0.52500000000000002</v>
+        <v>0.48799999999999999</v>
       </c>
       <c r="N43" s="9">
-        <v>0.5</v>
+        <v>0.41299999999999998</v>
       </c>
       <c r="O43" s="9">
-        <v>0.50900000000000001</v>
-      </c>
-      <c r="P43" s="28">
-        <v>0.51200000000000001</v>
+        <v>0.439</v>
+      </c>
+      <c r="P43" s="9">
+        <v>0.44700000000000001</v>
       </c>
       <c r="Q43" s="9">
-        <v>0.51500000000000001</v>
-      </c>
-    </row>
-    <row r="44" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.45600000000000002</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A44" s="21" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B44">
         <v>1</v>
@@ -8842,7 +8835,7 @@
         <v>0.5</v>
       </c>
       <c r="D44" s="21" t="s">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="E44">
         <v>60</v>
@@ -8850,41 +8843,41 @@
       <c r="F44">
         <v>132</v>
       </c>
-      <c r="G44" s="1">
-        <v>0.35</v>
-      </c>
-      <c r="H44" s="21"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="21" t="s">
+        <v>10</v>
+      </c>
       <c r="I44" s="7">
-        <v>355</v>
+        <v>248</v>
       </c>
       <c r="J44" s="7">
-        <v>323</v>
+        <v>430</v>
       </c>
       <c r="K44" s="7">
-        <v>370</v>
+        <v>187</v>
       </c>
       <c r="L44" s="8">
         <v>678</v>
       </c>
       <c r="M44" s="9">
-        <v>0.52400000000000002</v>
+        <v>0.36599999999999999</v>
       </c>
       <c r="N44" s="9">
-        <v>0.49</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="O44" s="9">
-        <v>0.502</v>
+        <v>0.46800000000000003</v>
       </c>
       <c r="P44" s="9">
-        <v>0.50600000000000001</v>
+        <v>0.44600000000000001</v>
       </c>
       <c r="Q44" s="9">
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="45" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.42499999999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A45" s="21" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B45">
         <v>1</v>
@@ -8893,7 +8886,7 @@
         <v>0.5</v>
       </c>
       <c r="D45" s="21" t="s">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E45">
         <v>60</v>
@@ -8901,41 +8894,41 @@
       <c r="F45">
         <v>132</v>
       </c>
-      <c r="G45" s="1">
-        <v>0.35</v>
-      </c>
-      <c r="H45" s="21"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="21" t="s">
+        <v>10</v>
+      </c>
       <c r="I45" s="7">
-        <v>360</v>
+        <v>248</v>
       </c>
       <c r="J45" s="7">
-        <v>318</v>
+        <v>430</v>
       </c>
       <c r="K45" s="7">
-        <v>440</v>
+        <v>187</v>
       </c>
       <c r="L45" s="8">
         <v>678</v>
       </c>
       <c r="M45" s="9">
-        <v>0.53100000000000003</v>
+        <v>0.36599999999999999</v>
       </c>
       <c r="N45" s="9">
-        <v>0.45</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="O45" s="9">
-        <v>0.47799999999999998</v>
+        <v>0.46800000000000003</v>
       </c>
       <c r="P45" s="9">
-        <v>0.48699999999999999</v>
+        <v>0.44600000000000001</v>
       </c>
       <c r="Q45" s="9">
-        <v>0.496</v>
-      </c>
-    </row>
-    <row r="46" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.42499999999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A46" s="21" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B46">
         <v>1</v>
@@ -8952,41 +8945,41 @@
       <c r="F46">
         <v>132</v>
       </c>
-      <c r="G46" s="1">
-        <v>0.35</v>
-      </c>
-      <c r="H46" s="21"/>
-      <c r="I46" s="30">
-        <v>373</v>
-      </c>
-      <c r="J46" s="30">
-        <v>305</v>
+      <c r="G46" s="1"/>
+      <c r="H46" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="I46" s="7">
+        <v>248</v>
+      </c>
+      <c r="J46" s="7">
+        <v>430</v>
       </c>
       <c r="K46" s="7">
-        <v>484</v>
+        <v>187</v>
       </c>
       <c r="L46" s="8">
         <v>678</v>
       </c>
-      <c r="M46" s="28">
-        <v>0.55000000000000004</v>
+      <c r="M46" s="9">
+        <v>0.36599999999999999</v>
       </c>
       <c r="N46" s="9">
-        <v>0.435</v>
-      </c>
-      <c r="O46" s="29">
-        <v>0.47399999999999998</v>
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="O46" s="9">
+        <v>0.46800000000000003</v>
       </c>
       <c r="P46" s="9">
-        <v>0.48599999999999999</v>
+        <v>0.44600000000000001</v>
       </c>
       <c r="Q46" s="9">
-        <v>0.499</v>
-      </c>
-    </row>
-    <row r="47" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.42499999999999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A47" s="21" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B47">
         <v>1</v>
@@ -8995,7 +8988,7 @@
         <v>0.5</v>
       </c>
       <c r="D47" s="21" t="s">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="E47">
         <v>60</v>
@@ -9004,40 +8997,40 @@
         <v>132</v>
       </c>
       <c r="G47" s="1">
-        <v>0.22500000000000001</v>
+        <v>0.65</v>
       </c>
       <c r="H47" s="21"/>
       <c r="I47" s="7">
-        <v>372</v>
+        <v>255</v>
       </c>
       <c r="J47" s="7">
-        <v>306</v>
+        <v>423</v>
       </c>
       <c r="K47" s="7">
-        <v>409</v>
+        <v>111</v>
       </c>
       <c r="L47" s="8">
         <v>678</v>
       </c>
       <c r="M47" s="9">
-        <v>0.54900000000000004</v>
+        <v>0.376</v>
       </c>
       <c r="N47" s="9">
-        <v>0.47599999999999998</v>
+        <v>0.69699999999999995</v>
       </c>
       <c r="O47" s="9">
-        <v>0.502</v>
+        <v>0.52300000000000002</v>
       </c>
       <c r="P47" s="9">
-        <v>0.51</v>
-      </c>
-      <c r="Q47" s="28">
-        <v>0.51800000000000002</v>
-      </c>
-    </row>
-    <row r="48" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.48899999999999999</v>
+      </c>
+      <c r="Q47" s="9">
+        <v>0.45800000000000002</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A48" s="21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B48">
         <v>1</v>
@@ -9046,7 +9039,7 @@
         <v>0.5</v>
       </c>
       <c r="D48" s="21" t="s">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E48">
         <v>60</v>
@@ -9055,40 +9048,40 @@
         <v>132</v>
       </c>
       <c r="G48" s="1">
-        <v>0.375</v>
+        <v>0.4</v>
       </c>
       <c r="H48" s="21"/>
       <c r="I48" s="7">
-        <v>324</v>
+        <v>305</v>
       </c>
       <c r="J48" s="7">
-        <v>354</v>
+        <v>373</v>
       </c>
       <c r="K48" s="7">
-        <v>428</v>
+        <v>233</v>
       </c>
       <c r="L48" s="8">
         <v>678</v>
       </c>
       <c r="M48" s="9">
-        <v>0.47799999999999998</v>
+        <v>0.45</v>
       </c>
       <c r="N48" s="9">
-        <v>0.43099999999999999</v>
+        <v>0.56699999999999995</v>
       </c>
       <c r="O48" s="9">
-        <v>0.44800000000000001</v>
+        <v>0.51500000000000001</v>
       </c>
       <c r="P48" s="9">
-        <v>0.45300000000000001</v>
+        <v>0.502</v>
       </c>
       <c r="Q48" s="9">
-        <v>0.45800000000000002</v>
-      </c>
-    </row>
-    <row r="49" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.48899999999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A49" s="21" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B49">
         <v>1</v>
@@ -9105,41 +9098,41 @@
       <c r="F49">
         <v>132</v>
       </c>
-      <c r="G49" s="1"/>
-      <c r="H49" s="21" t="s">
-        <v>26</v>
-      </c>
+      <c r="G49" s="1">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="H49" s="21"/>
       <c r="I49" s="7">
-        <v>331</v>
+        <v>367</v>
       </c>
       <c r="J49" s="7">
-        <v>347</v>
+        <v>311</v>
       </c>
       <c r="K49" s="7">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="L49" s="8">
         <v>678</v>
       </c>
       <c r="M49" s="9">
-        <v>0.48799999999999999</v>
+        <v>0.54100000000000004</v>
       </c>
       <c r="N49" s="9">
-        <v>0.41299999999999998</v>
+        <v>0.44</v>
       </c>
       <c r="O49" s="9">
-        <v>0.439</v>
+        <v>0.47399999999999998</v>
       </c>
       <c r="P49" s="9">
-        <v>0.44700000000000001</v>
+        <v>0.48499999999999999</v>
       </c>
       <c r="Q49" s="9">
-        <v>0.45600000000000002</v>
-      </c>
-    </row>
-    <row r="50" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.496</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A50" s="21" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B50">
         <v>1</v>
@@ -9148,7 +9141,7 @@
         <v>0.5</v>
       </c>
       <c r="D50" s="21" t="s">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="E50">
         <v>60</v>
@@ -9156,41 +9149,41 @@
       <c r="F50">
         <v>132</v>
       </c>
-      <c r="G50" s="1"/>
-      <c r="H50" s="21" t="s">
-        <v>10</v>
-      </c>
+      <c r="G50" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="H50" s="21"/>
       <c r="I50" s="7">
-        <v>248</v>
+        <v>269</v>
       </c>
       <c r="J50" s="7">
-        <v>430</v>
-      </c>
-      <c r="K50" s="7">
-        <v>187</v>
+        <v>409</v>
+      </c>
+      <c r="K50" s="30">
+        <v>164</v>
       </c>
       <c r="L50" s="8">
         <v>678</v>
       </c>
       <c r="M50" s="9">
-        <v>0.36599999999999999</v>
-      </c>
-      <c r="N50" s="9">
-        <v>0.56999999999999995</v>
+        <v>0.39700000000000002</v>
+      </c>
+      <c r="N50" s="28">
+        <v>0.621</v>
       </c>
       <c r="O50" s="9">
-        <v>0.46800000000000003</v>
-      </c>
-      <c r="P50" s="9">
-        <v>0.44600000000000001</v>
-      </c>
-      <c r="Q50" s="9">
-        <v>0.42499999999999999</v>
-      </c>
-    </row>
-    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.50900000000000001</v>
+      </c>
+      <c r="P50" s="29">
+        <v>0.48399999999999999</v>
+      </c>
+      <c r="Q50" s="39">
+        <v>0.46200000000000002</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A51" s="21" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B51">
         <v>1</v>
@@ -9199,7 +9192,7 @@
         <v>0.5</v>
       </c>
       <c r="D51" s="21" t="s">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E51">
         <v>60</v>
@@ -9208,38 +9201,38 @@
         <v>132</v>
       </c>
       <c r="G51" s="1">
-        <v>0.22500000000000001</v>
+        <v>0.4</v>
       </c>
       <c r="H51" s="21"/>
       <c r="I51" s="7">
-        <v>367</v>
+        <v>345</v>
       </c>
       <c r="J51" s="7">
-        <v>311</v>
+        <v>333</v>
       </c>
       <c r="K51" s="7">
-        <v>468</v>
+        <v>386</v>
       </c>
       <c r="L51" s="8">
         <v>678</v>
       </c>
       <c r="M51" s="9">
-        <v>0.54100000000000004</v>
+        <v>0.50900000000000001</v>
       </c>
       <c r="N51" s="9">
-        <v>0.44</v>
+        <v>0.47199999999999998</v>
       </c>
       <c r="O51" s="9">
-        <v>0.47399999999999998</v>
+        <v>0.48599999999999999</v>
       </c>
       <c r="P51" s="9">
-        <v>0.48499999999999999</v>
+        <v>0.49</v>
       </c>
       <c r="Q51" s="9">
-        <v>0.496</v>
-      </c>
-    </row>
-    <row r="52" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.49399999999999999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="21" t="s">
         <v>24</v>
       </c>
@@ -9290,9 +9283,9 @@
         <v>0.42899999999999999</v>
       </c>
     </row>
-    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A53" s="21" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B53">
         <v>1</v>
@@ -9301,7 +9294,7 @@
         <v>0.5</v>
       </c>
       <c r="D53" s="21" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="E53">
         <v>60</v>
@@ -9309,39 +9302,39 @@
       <c r="F53">
         <v>132</v>
       </c>
-      <c r="G53" s="1"/>
-      <c r="H53" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="I53" s="7">
-        <v>248</v>
-      </c>
-      <c r="J53" s="7">
-        <v>430</v>
+      <c r="G53" s="1">
+        <v>0.35</v>
+      </c>
+      <c r="H53" s="21"/>
+      <c r="I53" s="30">
+        <v>373</v>
+      </c>
+      <c r="J53" s="30">
+        <v>305</v>
       </c>
       <c r="K53" s="7">
-        <v>187</v>
+        <v>484</v>
       </c>
       <c r="L53" s="8">
         <v>678</v>
       </c>
-      <c r="M53" s="9">
-        <v>0.36599999999999999</v>
+      <c r="M53" s="28">
+        <v>0.55000000000000004</v>
       </c>
       <c r="N53" s="9">
-        <v>0.56999999999999995</v>
-      </c>
-      <c r="O53" s="9">
-        <v>0.46800000000000003</v>
+        <v>0.435</v>
+      </c>
+      <c r="O53" s="29">
+        <v>0.47399999999999998</v>
       </c>
       <c r="P53" s="9">
-        <v>0.44600000000000001</v>
+        <v>0.48599999999999999</v>
       </c>
       <c r="Q53" s="9">
-        <v>0.42499999999999999</v>
-      </c>
-    </row>
-    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.499</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="21" t="s">
         <v>21</v>
       </c>
@@ -9392,9 +9385,9 @@
         <v>0.41599999999999998</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A55" s="21" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="B55">
         <v>1</v>
@@ -9412,38 +9405,38 @@
         <v>132</v>
       </c>
       <c r="G55" s="1">
-        <v>0.65</v>
+        <v>0.4</v>
       </c>
       <c r="H55" s="21"/>
       <c r="I55" s="7">
-        <v>255</v>
+        <v>299</v>
       </c>
       <c r="J55" s="7">
-        <v>423</v>
+        <v>379</v>
       </c>
       <c r="K55" s="7">
-        <v>111</v>
+        <v>193</v>
       </c>
       <c r="L55" s="8">
         <v>678</v>
       </c>
-      <c r="M55" s="9">
-        <v>0.376</v>
+      <c r="M55" s="36">
+        <v>0.441</v>
       </c>
       <c r="N55" s="9">
-        <v>0.69699999999999995</v>
-      </c>
-      <c r="O55" s="9">
-        <v>0.52300000000000002</v>
-      </c>
-      <c r="P55" s="9">
-        <v>0.48899999999999999</v>
-      </c>
-      <c r="Q55" s="9">
-        <v>0.45800000000000002</v>
-      </c>
-    </row>
-    <row r="56" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.60799999999999998</v>
+      </c>
+      <c r="O55" s="28">
+        <v>0.53</v>
+      </c>
+      <c r="P55" s="28">
+        <v>0.51100000000000001</v>
+      </c>
+      <c r="Q55" s="36">
+        <v>0.49399999999999999</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="21" t="s">
         <v>22</v>
       </c>
@@ -9494,9 +9487,9 @@
         <v>0.46300000000000002</v>
       </c>
     </row>
-    <row r="57" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A57" s="21" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="B57">
         <v>1</v>
@@ -9505,7 +9498,7 @@
         <v>0.5</v>
       </c>
       <c r="D57" s="21" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E57">
         <v>60</v>
@@ -9514,38 +9507,38 @@
         <v>132</v>
       </c>
       <c r="G57" s="1">
-        <v>0.65</v>
+        <v>0.25</v>
       </c>
       <c r="H57" s="21"/>
       <c r="I57" s="7">
-        <v>269</v>
+        <v>356</v>
       </c>
       <c r="J57" s="7">
-        <v>409</v>
-      </c>
-      <c r="K57" s="30">
-        <v>164</v>
+        <v>322</v>
+      </c>
+      <c r="K57" s="7">
+        <v>356</v>
       </c>
       <c r="L57" s="8">
         <v>678</v>
       </c>
       <c r="M57" s="9">
-        <v>0.39700000000000002</v>
-      </c>
-      <c r="N57" s="28">
-        <v>0.621</v>
+        <v>0.52500000000000002</v>
+      </c>
+      <c r="N57" s="9">
+        <v>0.5</v>
       </c>
       <c r="O57" s="9">
         <v>0.50900000000000001</v>
       </c>
-      <c r="P57" s="29">
-        <v>0.48399999999999999</v>
-      </c>
-      <c r="Q57" s="39">
-        <v>0.46200000000000002</v>
-      </c>
-    </row>
-    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P57" s="28">
+        <v>0.51200000000000001</v>
+      </c>
+      <c r="Q57" s="9">
+        <v>0.51500000000000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="21" t="s">
         <v>17</v>
       </c>
@@ -9598,7 +9591,7 @@
         <v>0.42599999999999999</v>
       </c>
     </row>
-    <row r="59" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A59" s="21" t="s">
         <v>2</v>
       </c>
@@ -9609,7 +9602,7 @@
         <v>0.5</v>
       </c>
       <c r="D59" s="21" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="E59">
         <v>60</v>
@@ -9618,38 +9611,38 @@
         <v>132</v>
       </c>
       <c r="G59" s="1">
-        <v>0.4</v>
+        <v>0.22500000000000001</v>
       </c>
       <c r="H59" s="21"/>
       <c r="I59" s="7">
-        <v>299</v>
+        <v>372</v>
       </c>
       <c r="J59" s="7">
-        <v>379</v>
+        <v>306</v>
       </c>
       <c r="K59" s="7">
-        <v>193</v>
+        <v>409</v>
       </c>
       <c r="L59" s="8">
         <v>678</v>
       </c>
-      <c r="M59" s="36">
-        <v>0.441</v>
+      <c r="M59" s="9">
+        <v>0.54900000000000004</v>
       </c>
       <c r="N59" s="9">
-        <v>0.60799999999999998</v>
-      </c>
-      <c r="O59" s="28">
-        <v>0.53</v>
-      </c>
-      <c r="P59" s="28">
-        <v>0.51100000000000001</v>
-      </c>
-      <c r="Q59" s="36">
-        <v>0.49399999999999999</v>
-      </c>
-    </row>
-    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+        <v>0.47599999999999998</v>
+      </c>
+      <c r="O59" s="9">
+        <v>0.502</v>
+      </c>
+      <c r="P59" s="9">
+        <v>0.51</v>
+      </c>
+      <c r="Q59" s="28">
+        <v>0.51800000000000002</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="21" t="s">
         <v>2</v>
       </c>
@@ -9700,7 +9693,7 @@
         <v>0.45400000000000001</v>
       </c>
     </row>
-    <row r="61" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="21" t="s">
         <v>3</v>
       </c>
@@ -9751,7 +9744,7 @@
         <v>0.503</v>
       </c>
     </row>
-    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="21" t="s">
         <v>16</v>
       </c>
@@ -9804,7 +9797,7 @@
         <v>0.47299999999999998</v>
       </c>
     </row>
-    <row r="63" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="21" t="s">
         <v>17</v>
       </c>
@@ -9857,7 +9850,7 @@
         <v>0.46899999999999997</v>
       </c>
     </row>
-    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="21" t="s">
         <v>2</v>
       </c>
@@ -9908,7 +9901,7 @@
         <v>0.47799999999999998</v>
       </c>
     </row>
-    <row r="65" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="21" t="s">
         <v>23</v>
       </c>
@@ -9959,7 +9952,7 @@
         <v>0.45700000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="21" t="s">
         <v>24</v>
       </c>
@@ -10010,7 +10003,7 @@
         <v>0.437</v>
       </c>
     </row>
-    <row r="67" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="21" t="s">
         <v>21</v>
       </c>
@@ -10061,7 +10054,7 @@
         <v>0.41599999999999998</v>
       </c>
     </row>
-    <row r="68" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="21" t="s">
         <v>22</v>
       </c>
@@ -10112,7 +10105,7 @@
         <v>0.47899999999999998</v>
       </c>
     </row>
-    <row r="69" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="21" t="s">
         <v>3</v>
       </c>
@@ -10163,7 +10156,7 @@
         <v>0.503</v>
       </c>
     </row>
-    <row r="70" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="21" t="s">
         <v>16</v>
       </c>
@@ -10216,7 +10209,7 @@
         <v>0.47299999999999998</v>
       </c>
     </row>
-    <row r="71" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="21" t="s">
         <v>17</v>
       </c>
@@ -10269,7 +10262,7 @@
         <v>0.47499999999999998</v>
       </c>
     </row>
-    <row r="72" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="21" t="s">
         <v>2</v>
       </c>
@@ -10320,7 +10313,7 @@
         <v>0.49399999999999999</v>
       </c>
     </row>
-    <row r="73" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="21" t="s">
         <v>23</v>
       </c>
@@ -10371,7 +10364,7 @@
         <v>0.45800000000000002</v>
       </c>
     </row>
-    <row r="74" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="21" t="s">
         <v>24</v>
       </c>
@@ -10422,7 +10415,7 @@
         <v>0.44600000000000001</v>
       </c>
     </row>
-    <row r="75" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="21" t="s">
         <v>21</v>
       </c>
@@ -10473,7 +10466,7 @@
         <v>0.41599999999999998</v>
       </c>
     </row>
-    <row r="76" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="21" t="s">
         <v>22</v>
       </c>
@@ -10524,7 +10517,7 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="77" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="34" t="s">
         <v>3</v>
       </c>
@@ -10577,7 +10570,7 @@
         <v>0.216</v>
       </c>
     </row>
-    <row r="78" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="21" t="s">
         <v>3</v>
       </c>
@@ -10628,7 +10621,7 @@
         <v>0.26100000000000001</v>
       </c>
     </row>
-    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="21" t="s">
         <v>16</v>
       </c>
@@ -10679,7 +10672,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="80" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="21" t="s">
         <v>17</v>
       </c>
@@ -10730,7 +10723,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="81" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="21" t="s">
         <v>2</v>
       </c>
@@ -10781,7 +10774,7 @@
         <v>0.32400000000000001</v>
       </c>
     </row>
-    <row r="82" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="21" t="s">
         <v>24</v>
       </c>
@@ -10832,7 +10825,7 @@
         <v>0.27400000000000002</v>
       </c>
     </row>
-    <row r="83" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="21" t="s">
         <v>21</v>
       </c>
@@ -10883,7 +10876,7 @@
         <v>0.22800000000000001</v>
       </c>
     </row>
-    <row r="84" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="21" t="s">
         <v>22</v>
       </c>
@@ -10934,7 +10927,7 @@
         <v>0.316</v>
       </c>
     </row>
-    <row r="85" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="21" t="s">
         <v>3</v>
       </c>
@@ -10985,7 +10978,7 @@
         <v>0.32700000000000001</v>
       </c>
     </row>
-    <row r="86" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="21" t="s">
         <v>16</v>
       </c>
@@ -11038,7 +11031,7 @@
         <v>0.33300000000000002</v>
       </c>
     </row>
-    <row r="87" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="21" t="s">
         <v>17</v>
       </c>
@@ -11091,7 +11084,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="88" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="21" t="s">
         <v>2</v>
       </c>
@@ -11142,7 +11135,7 @@
         <v>0.32400000000000001</v>
       </c>
     </row>
-    <row r="89" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="21" t="s">
         <v>24</v>
       </c>
@@ -11193,7 +11186,7 @@
         <v>0.27400000000000002</v>
       </c>
     </row>
-    <row r="90" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="21" t="s">
         <v>21</v>
       </c>
@@ -11244,7 +11237,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="91" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="21" t="s">
         <v>22</v>
       </c>
@@ -11295,7 +11288,7 @@
         <v>0.316</v>
       </c>
     </row>
-    <row r="92" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="21" t="s">
         <v>3</v>
       </c>
@@ -11346,7 +11339,7 @@
         <v>0.32700000000000001</v>
       </c>
     </row>
-    <row r="93" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="21" t="s">
         <v>16</v>
       </c>
@@ -11399,7 +11392,7 @@
         <v>0.33300000000000002</v>
       </c>
     </row>
-    <row r="94" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="21" t="s">
         <v>17</v>
       </c>
@@ -11452,7 +11445,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="95" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="21" t="s">
         <v>2</v>
       </c>
@@ -11503,7 +11496,7 @@
         <v>0.32800000000000001</v>
       </c>
     </row>
-    <row r="96" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="21" t="s">
         <v>24</v>
       </c>
@@ -11554,7 +11547,7 @@
         <v>0.27200000000000002</v>
       </c>
     </row>
-    <row r="97" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="21" t="s">
         <v>21</v>
       </c>
@@ -11603,7 +11596,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="98" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="21" t="s">
         <v>22</v>
       </c>
@@ -11654,7 +11647,7 @@
         <v>0.32300000000000001</v>
       </c>
     </row>
-    <row r="99" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="34" t="s">
         <v>3</v>
       </c>
@@ -11707,7 +11700,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="100" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="21" t="s">
         <v>3</v>
       </c>
@@ -11758,7 +11751,7 @@
         <v>0.252</v>
       </c>
     </row>
-    <row r="101" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="21" t="s">
         <v>16</v>
       </c>
@@ -11812,7 +11805,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="102" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="21" t="s">
         <v>17</v>
       </c>
@@ -11863,7 +11856,7 @@
         <v>0.24199999999999999</v>
       </c>
     </row>
-    <row r="103" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="21" t="s">
         <v>2</v>
       </c>
@@ -11914,7 +11907,7 @@
         <v>0.26100000000000001</v>
       </c>
     </row>
-    <row r="104" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="21" t="s">
         <v>21</v>
       </c>
@@ -11965,7 +11958,7 @@
         <v>0.221</v>
       </c>
     </row>
-    <row r="105" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="21" t="s">
         <v>22</v>
       </c>
@@ -12018,7 +12011,7 @@
         <v>0.27100000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="21" t="s">
         <v>3</v>
       </c>
@@ -12069,7 +12062,7 @@
         <v>0.252</v>
       </c>
     </row>
-    <row r="107" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="21" t="s">
         <v>16</v>
       </c>
@@ -12120,7 +12113,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="108" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="21" t="s">
         <v>17</v>
       </c>
@@ -12173,7 +12166,7 @@
         <v>0.23699999999999999</v>
       </c>
     </row>
-    <row r="109" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="21" t="s">
         <v>2</v>
       </c>
@@ -12226,7 +12219,7 @@
         <v>0.26600000000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="21" t="s">
         <v>21</v>
       </c>
@@ -12280,7 +12273,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="111" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="21" t="s">
         <v>22</v>
       </c>
@@ -12333,7 +12326,7 @@
         <v>0.26900000000000002</v>
       </c>
     </row>
-    <row r="112" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="21" t="s">
         <v>3</v>
       </c>
@@ -12384,7 +12377,7 @@
         <v>0.26400000000000001</v>
       </c>
     </row>
-    <row r="113" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="21" t="s">
         <v>16</v>
       </c>
@@ -12437,7 +12430,7 @@
         <v>0.26600000000000001</v>
       </c>
     </row>
-    <row r="114" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="21" t="s">
         <v>17</v>
       </c>
@@ -12490,7 +12483,7 @@
         <v>0.23699999999999999</v>
       </c>
     </row>
-    <row r="115" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="21" t="s">
         <v>2</v>
       </c>
@@ -12541,7 +12534,7 @@
         <v>0.26300000000000001</v>
       </c>
     </row>
-    <row r="116" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="21" t="s">
         <v>21</v>
       </c>
@@ -12595,7 +12588,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="117" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:19" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="21" t="s">
         <v>22</v>
       </c>
@@ -12648,27 +12641,27 @@
         <v>0.26900000000000002</v>
       </c>
     </row>
-    <row r="120" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A120" s="26" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="121" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A121" s="25" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="122" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A122" s="38" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="123" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A123" s="33" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>3</v>
       </c>
@@ -12715,7 +12708,7 @@
         <v>0.48899999999999999</v>
       </c>
     </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>3</v>
       </c>
@@ -12762,7 +12755,7 @@
         <v>0.48699999999999999</v>
       </c>
     </row>
-    <row r="128" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>16</v>
       </c>
@@ -12809,7 +12802,7 @@
         <v>0.47299999999999998</v>
       </c>
     </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>17</v>
       </c>
@@ -12856,7 +12849,7 @@
         <v>0.46200000000000002</v>
       </c>
     </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>2</v>
       </c>
@@ -12906,7 +12899,7 @@
         <v>0.49399999999999999</v>
       </c>
     </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>2</v>
       </c>
@@ -12947,7 +12940,7 @@
         <v>0.31900000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>2</v>
       </c>
@@ -12985,7 +12978,7 @@
         <v>0.504</v>
       </c>
     </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A138" s="21" t="s">
         <v>23</v>
       </c>
@@ -13033,7 +13026,7 @@
         <v>0.45700000000000002</v>
       </c>
     </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A139" s="21" t="s">
         <v>23</v>
       </c>
@@ -13081,7 +13074,7 @@
         <v>0.45700000000000002</v>
       </c>
     </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A141" s="21" t="s">
         <v>24</v>
       </c>
@@ -13129,7 +13122,7 @@
         <v>0.43</v>
       </c>
     </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A142" s="21" t="s">
         <v>24</v>
       </c>
@@ -13177,7 +13170,7 @@
         <v>0.42899999999999999</v>
       </c>
     </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A144" s="21" t="s">
         <v>21</v>
       </c>
@@ -13225,7 +13218,7 @@
         <v>0.42499999999999999</v>
       </c>
     </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A145" s="21" t="s">
         <v>21</v>
       </c>
@@ -13273,7 +13266,7 @@
         <v>0.41599999999999998</v>
       </c>
     </row>
-    <row r="147" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A147" s="21" t="s">
         <v>22</v>
       </c>
@@ -13321,7 +13314,7 @@
         <v>0.45800000000000002</v>
       </c>
     </row>
-    <row r="148" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A148" s="21" t="s">
         <v>22</v>
       </c>
@@ -13370,7 +13363,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="149" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A149" s="40" t="s">
         <v>22</v>
       </c>

</xml_diff>